<commit_message>
Add newsletter confirmation to site inventory
</commit_message>
<xml_diff>
--- a/jonathan-harris-site-url-inventory-remediated-release-ready.xlsx
+++ b/jonathan-harris-site-url-inventory-remediated-release-ready.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ebook Source of Truth" sheetId="1" r:id="R804034c698414f35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pages" sheetId="2" r:id="R4eaff81115304199"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R6f1f5247873143bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BuyNow Redirects" sheetId="4" r:id="R3ac8191d87ac441f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ebooks Master" sheetId="5" r:id="R8795a2f087244cba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ebook Source of Truth" sheetId="1" r:id="Rbe624c866a994b62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pages" sheetId="2" r:id="R9d1b23a1e1cf4221"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Rfd3d444b0850455f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BuyNow Redirects" sheetId="4" r:id="R044d5f2de11e4125"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ebooks Master" sheetId="5" r:id="R9fc73bbfe0814cf7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -151,10 +151,11 @@
     <x:border/>
     <x:border/>
   </x:borders>
-  <x:cellStyleXfs count="1">
+  <x:cellStyleXfs count="2">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="79">
+  <x:cellXfs count="86">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="bottom"/>
     </x:xf>
@@ -357,6 +358,27 @@
     <x:xf numFmtId="0" fontId="11" fillId="3" borderId="6" xfId="0"/>
     <x:xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="1" fontId="2" fillId="0" borderId="3" xfId="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="2" fillId="0" borderId="3" xfId="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -8865,18 +8887,28 @@
       <x:c r="Z91" s="46" t="n"/>
     </x:row>
     <x:row r="92" s="72" customFormat="1" ht="21" customHeight="1">
-      <x:c r="A92" s="46" t="n"/>
-      <x:c r="B92" s="46" t="n"/>
-      <x:c r="C92" s="46" t="n"/>
-      <x:c r="D92" s="46" t="n"/>
-      <x:c r="E92" s="46" t="n"/>
-      <x:c r="F92" s="46" t="n"/>
-      <x:c r="G92" s="46" t="n"/>
-      <x:c r="H92" s="46" t="n"/>
-      <x:c r="I92" s="46" t="n"/>
-      <x:c r="J92" s="46" t="n"/>
-      <x:c r="K92" s="46" t="n"/>
-      <x:c r="L92" s="46" t="n"/>
+      <x:c r="A92" s="79" t="str">
+        <x:v>newsletter/thanks/index.html</x:v>
+      </x:c>
+      <x:c r="B92" s="80" t="str">
+        <x:v>/newsletter/thanks/</x:v>
+      </x:c>
+      <x:c r="C92" s="81" t="str">
+        <x:v>https://jonathan-harris.online/newsletter/thanks/</x:v>
+      </x:c>
+      <x:c r="D92" s="82" t="str">
+        <x:v>Thanks for signing up | AI Edge</x:v>
+      </x:c>
+      <x:c r="E92" s="82" t="str">
+        <x:v>Standard page route</x:v>
+      </x:c>
+      <x:c r="F92" s="83"/>
+      <x:c r="G92" s="83"/>
+      <x:c r="H92" s="82"/>
+      <x:c r="I92" s="82"/>
+      <x:c r="J92" s="84"/>
+      <x:c r="K92" s="85"/>
+      <x:c r="L92" s="83"/>
       <x:c r="M92" s="46" t="n"/>
       <x:c r="N92" s="46" t="n"/>
       <x:c r="O92" s="46" t="n"/>
@@ -15440,7 +15472,7 @@
       </x:c>
       <x:c r="B4" s="65" t="n">
         <x:f>COUNTA(Pages!A6:A200)</x:f>
-        <x:v>86</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="C4" s="42" t="n"/>
       <x:c r="D4" s="42" t="n"/>

</xml_diff>